<commit_message>
test(calculators): tests for 6.4.1.1 crop burning n20
test(calculators): adding tests for 6.4.1.1 crop burning ch4

test(calculators): adding tests for 6.3.1.1 crop and pasture residues

feat(calculators): :art: implement 6.2.1.1 method 2, with tests for m1 and m2
</commit_message>
<xml_diff>
--- a/packages/calculators/src/modules/test/6.1-crop-residues.xlsx
+++ b/packages/calculators/src/modules/test/6.1-crop-residues.xlsx
@@ -8,13 +8,12 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/eddiesholl/Code/aginnovationaustralia/emissions-calculators/packages/calculators/src/modules/test/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{30571FFF-B9A4-BC4C-ABDA-D344413820C7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CE1AC328-8952-844F-ACEA-695B8035CAFF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="51200" yWindow="11440" windowWidth="28800" windowHeight="23520" xr2:uid="{5678E890-3691-CF46-80E7-00FB1F103661}"/>
+    <workbookView xWindow="51200" yWindow="-5540" windowWidth="28800" windowHeight="23520" xr2:uid="{5678E890-3691-CF46-80E7-00FB1F103661}"/>
   </bookViews>
   <sheets>
     <sheet name="6.1.1.1" sheetId="1" r:id="rId1"/>
-    <sheet name="5.4.1.3" sheetId="2" r:id="rId2"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -37,7 +36,7 @@
 </file>
 
 <file path=xl/metadata.xml><?xml version="1.0" encoding="utf-8"?>
-<metadata xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xlrd="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata" xmlns:xda="http://schemas.microsoft.com/office/spreadsheetml/2017/dynamicarray">
+<metadata xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xda="http://schemas.microsoft.com/office/spreadsheetml/2017/dynamicarray">
   <metadataTypes count="1">
     <metadataType name="XLDAPR" minSupportedVersion="120000" copy="1" pasteAll="1" pasteValues="1" merge="1" splitFirst="1" rowColShift="1" clearFormats="1" clearComments="1" assign="1" coerce="1" cellMeta="1"/>
   </metadataTypes>
@@ -59,7 +58,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="196" uniqueCount="115">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="148" uniqueCount="73">
   <si>
     <t>Method 1</t>
   </si>
@@ -70,283 +69,7 @@
     <t>Cn2o</t>
   </si>
   <si>
-    <t>Table A.2.2.3</t>
-  </si>
-  <si>
-    <t>Irrigated pasture</t>
-  </si>
-  <si>
-    <t>Irrigated crop (low rainfall)</t>
-  </si>
-  <si>
-    <t>Irrigated crop (high rainfall)</t>
-  </si>
-  <si>
-    <t>Irrigated crop</t>
-  </si>
-  <si>
-    <t>Non-irrigated pasture</t>
-  </si>
-  <si>
-    <t>Non-irrigated crops</t>
-  </si>
-  <si>
-    <t>Sugar</t>
-  </si>
-  <si>
     <t>Cotton</t>
-  </si>
-  <si>
-    <t>Horticultural crops</t>
-  </si>
-  <si>
-    <t>Aquaculture</t>
-  </si>
-  <si>
-    <t>Rice (continuous flooding)</t>
-  </si>
-  <si>
-    <t>Rice (single and multiple drainage, or alternate wetting and drying)</t>
-  </si>
-  <si>
-    <t>Forestry</t>
-  </si>
-  <si>
-    <t>EFn2oj</t>
-  </si>
-  <si>
-    <t>Production system</t>
-  </si>
-  <si>
-    <t>TMjf</t>
-  </si>
-  <si>
-    <t>Fnorganicf</t>
-  </si>
-  <si>
-    <t>Custom Fnorganic</t>
-  </si>
-  <si>
-    <t>Type</t>
-  </si>
-  <si>
-    <t>Table A.2.2.6</t>
-  </si>
-  <si>
-    <t>Monoammonium phosphate (MAP)</t>
-  </si>
-  <si>
-    <t>Diammonium phosphate (DAP)</t>
-  </si>
-  <si>
-    <t>Urea</t>
-  </si>
-  <si>
-    <t>Sulphate of Ammonia (SOA)</t>
-  </si>
-  <si>
-    <t>Ammonium nitrate (AN)</t>
-  </si>
-  <si>
-    <t>Urea-based fertilisers </t>
-  </si>
-  <si>
-    <t>Ammonium-based fertilisers </t>
-  </si>
-  <si>
-    <t>Nitrate-based fertilisers </t>
-  </si>
-  <si>
-    <t>Ammonium-nitrate based fertilisers </t>
-  </si>
-  <si>
-    <t>Other fertilisers </t>
-  </si>
-  <si>
-    <t>Table A.2.2.9</t>
-  </si>
-  <si>
-    <t>Total mass applied in kg</t>
-  </si>
-  <si>
-    <t>Note that Table A.2.2.9 has been mapped to A.2.2.6, pending approval</t>
-  </si>
-  <si>
-    <t>Calcium Ammonium Nitrate (CAN)</t>
-  </si>
-  <si>
-    <t>Urea-Ammonium Nitrate (UAN)</t>
-  </si>
-  <si>
-    <r>
-      <t>𝐸</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="8"/>
-        <color rgb="FF000000"/>
-        <rFont val="Helvetica"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">𝑎𝑑,𝑜𝑟𝑔𝑎𝑛𝑖𝑐 </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF000000"/>
-        <rFont val="Helvetica"/>
-        <family val="2"/>
-      </rPr>
-      <t>= ∑ ∑ (𝑀</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="8"/>
-        <color rgb="FF000000"/>
-        <rFont val="Helvetica"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">𝑣𝑜𝑙,𝑜𝑟𝑔𝑎𝑛𝑖𝑐,𝑗𝑓 </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF000000"/>
-        <rFont val="Helvetica"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">× 𝐸𝐹 </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="8"/>
-        <color rgb="FF000000"/>
-        <rFont val="Helvetica"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">𝑁2𝑂,𝑗 </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF000000"/>
-        <rFont val="Helvetica"/>
-        <family val="2"/>
-      </rPr>
-      <t>× 𝐶</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="8"/>
-        <color rgb="FF000000"/>
-        <rFont val="Helvetica"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">𝑁2𝑂 </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF000000"/>
-        <rFont val="Helvetica"/>
-        <family val="2"/>
-      </rPr>
-      <t>× 10</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="8"/>
-        <color rgb="FF000000"/>
-        <rFont val="Helvetica"/>
-        <family val="2"/>
-      </rPr>
-      <t>−3</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF000000"/>
-        <rFont val="Helvetica"/>
-        <family val="2"/>
-      </rPr>
-      <t>)</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <t>𝑀</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="8"/>
-        <color rgb="FF000000"/>
-        <rFont val="Helvetica"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">𝑣𝑜𝑙,𝑜𝑟𝑔𝑎𝑛𝑖𝑐,𝑗𝑓 </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF000000"/>
-        <rFont val="Helvetica"/>
-        <family val="2"/>
-      </rPr>
-      <t>= 𝑀𝑁𝑆𝑜𝑖𝑙</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="8"/>
-        <color rgb="FF000000"/>
-        <rFont val="Helvetica"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">𝑗𝑓 </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF000000"/>
-        <rFont val="Helvetica"/>
-        <family val="2"/>
-      </rPr>
-      <t>× 𝐹𝑟𝑎𝑐𝐺𝐴𝑆𝑀</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="8"/>
-        <color rgb="FF000000"/>
-        <rFont val="Helvetica"/>
-        <family val="2"/>
-      </rPr>
-      <t>𝑠𝑜𝑖𝑙</t>
-    </r>
-  </si>
-  <si>
-    <t>Mvolorganic</t>
-  </si>
-  <si>
-    <r>
-      <t>FracGASM</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="6"/>
-        <color rgb="FF000000"/>
-        <rFont val="Arial"/>
-        <family val="2"/>
-      </rPr>
-      <t>soil</t>
-    </r>
-  </si>
-  <si>
-    <t>MNSoiljf</t>
-  </si>
-  <si>
-    <t>TODO: MNSoil blocked on NTjmt2</t>
-  </si>
-  <si>
-    <t>Eadorganic</t>
   </si>
   <si>
     <t>E</t>
@@ -853,10 +576,10 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <numFmts count="2">
-    <numFmt numFmtId="167" formatCode="0.000"/>
-    <numFmt numFmtId="168" formatCode="0.0000"/>
+    <numFmt numFmtId="164" formatCode="0.000"/>
+    <numFmt numFmtId="165" formatCode="0.0000"/>
   </numFmts>
-  <fonts count="9">
+  <fonts count="8">
     <font>
       <sz val="12"/>
       <color theme="1"/>
@@ -901,12 +624,6 @@
       <family val="2"/>
     </font>
     <font>
-      <sz val="6"/>
-      <color rgb="FF000000"/>
-      <name val="Arial"/>
-      <family val="2"/>
-    </font>
-    <font>
       <sz val="12"/>
       <color rgb="FF000000"/>
       <name val="Helvetica"/>
@@ -945,7 +662,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="17">
+  <cellXfs count="15">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -958,17 +675,15 @@
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="2" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="167" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="168" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="167" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="164" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="165" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1323,7 +1038,7 @@
     <col min="16" max="16" width="12.83203125" customWidth="1"/>
     <col min="18" max="18" width="12.1640625" bestFit="1" customWidth="1"/>
     <col min="20" max="20" width="36" customWidth="1"/>
-    <col min="24" max="24" width="6.33203125" style="10" bestFit="1" customWidth="1"/>
+    <col min="24" max="24" width="6.33203125" style="8" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:22" ht="17">
@@ -1331,7 +1046,7 @@
         <v>0</v>
       </c>
       <c r="R1" s="1" t="s">
-        <v>47</v>
+        <v>5</v>
       </c>
     </row>
     <row r="2" spans="1:22">
@@ -1339,83 +1054,81 @@
       <c r="R2" s="1"/>
     </row>
     <row r="3" spans="1:22" ht="34">
-      <c r="F3" s="10" t="s">
-        <v>98</v>
-      </c>
-      <c r="G3" s="10" t="s">
-        <v>108</v>
-      </c>
-      <c r="H3" s="10"/>
-      <c r="I3" s="10" t="s">
-        <v>109</v>
-      </c>
-      <c r="J3" s="10" t="s">
-        <v>112</v>
-      </c>
-      <c r="K3" s="10" t="s">
-        <v>110</v>
-      </c>
-      <c r="L3" s="10" t="s">
-        <v>111</v>
-      </c>
-      <c r="M3" s="10"/>
-      <c r="N3" s="10"/>
-      <c r="O3" s="10"/>
+      <c r="F3" s="8" t="s">
+        <v>56</v>
+      </c>
+      <c r="G3" s="8" t="s">
+        <v>66</v>
+      </c>
+      <c r="H3" s="8"/>
+      <c r="I3" s="8" t="s">
+        <v>67</v>
+      </c>
+      <c r="J3" s="8" t="s">
+        <v>70</v>
+      </c>
+      <c r="K3" s="8" t="s">
+        <v>68</v>
+      </c>
+      <c r="L3" s="8" t="s">
+        <v>69</v>
+      </c>
+      <c r="M3" s="8"/>
+      <c r="N3" s="8"/>
+      <c r="O3" s="8"/>
       <c r="P3" s="1" t="s">
-        <v>56</v>
+        <v>14</v>
       </c>
       <c r="R3" s="1"/>
     </row>
     <row r="4" spans="1:22" ht="17">
       <c r="A4" s="4" t="s">
-        <v>54</v>
+        <v>12</v>
       </c>
       <c r="B4" s="5" t="s">
-        <v>68</v>
+        <v>26</v>
       </c>
       <c r="C4" s="5" t="s">
-        <v>71</v>
+        <v>29</v>
       </c>
       <c r="D4" s="5" t="s">
-        <v>85</v>
+        <v>43</v>
       </c>
       <c r="E4" s="5" t="s">
-        <v>57</v>
+        <v>15</v>
       </c>
       <c r="F4" s="5" t="s">
-        <v>69</v>
-      </c>
-      <c r="G4" s="9" t="s">
-        <v>72</v>
-      </c>
-      <c r="H4" s="9" t="s">
-        <v>84</v>
-      </c>
-      <c r="I4" s="9" t="s">
-        <v>60</v>
-      </c>
-      <c r="J4" s="9" t="s">
-        <v>61</v>
-      </c>
-      <c r="K4" s="9" t="s">
-        <v>62</v>
-      </c>
-      <c r="L4" s="9" t="s">
-        <v>64</v>
-      </c>
-      <c r="M4" s="9"/>
-      <c r="N4" s="9" t="s">
-        <v>83</v>
-      </c>
-      <c r="O4" s="9"/>
+        <v>27</v>
+      </c>
+      <c r="G4" t="s">
+        <v>30</v>
+      </c>
+      <c r="H4" t="s">
+        <v>42</v>
+      </c>
+      <c r="I4" t="s">
+        <v>18</v>
+      </c>
+      <c r="J4" t="s">
+        <v>19</v>
+      </c>
+      <c r="K4" t="s">
+        <v>20</v>
+      </c>
+      <c r="L4" t="s">
+        <v>22</v>
+      </c>
+      <c r="N4" t="s">
+        <v>41</v>
+      </c>
       <c r="P4" t="s">
-        <v>55</v>
+        <v>13</v>
       </c>
       <c r="Q4" t="s">
-        <v>48</v>
+        <v>6</v>
       </c>
       <c r="R4" s="6" t="s">
-        <v>46</v>
+        <v>4</v>
       </c>
       <c r="T4" s="7" t="s">
         <v>1</v>
@@ -1423,13 +1136,13 @@
     </row>
     <row r="5" spans="1:22">
       <c r="A5" s="2" t="s">
-        <v>52</v>
+        <v>10</v>
       </c>
       <c r="B5" t="s">
-        <v>82</v>
+        <v>40</v>
       </c>
       <c r="C5" t="s">
-        <v>77</v>
+        <v>35</v>
       </c>
       <c r="D5">
         <v>50</v>
@@ -1437,67 +1150,67 @@
       <c r="E5">
         <v>2000</v>
       </c>
-      <c r="F5" s="16">
+      <c r="F5" s="14">
         <v>0.2</v>
       </c>
-      <c r="G5" s="16" cm="1">
+      <c r="G5" s="14" cm="1">
         <f t="array" ref="G5">_xlfn.IFS(ISBLANK(A5), "",B5="Sugar Cane", VLOOKUP(C5, $U$48:$V$50, 2, FALSE),_xlfn.IFNA(MATCH(B5, $T$43:$T$47, 0), FALSE), VLOOKUP(B5, $T$43:$V$47, 3, FALSE), TRUE, VLOOKUP(C5, $U$51:$V$53, 2, FALSE))</f>
         <v>0</v>
       </c>
-      <c r="H5" s="16">
-        <f>IF(ISBLANK(A5), "", D5*E5)</f>
+      <c r="H5" s="14">
+        <f t="shared" ref="H5:H14" si="0">IF(ISBLANK(A5), "", D5*E5)</f>
         <v>100000</v>
       </c>
-      <c r="I5" s="16">
-        <f>IF(ISBLANK($A5), "", VLOOKUP($B5, $T$22:$AB$39, 2, FALSE))</f>
+      <c r="I5" s="14">
+        <f t="shared" ref="I5:I14" si="1">IF(ISBLANK($A5), "", VLOOKUP($B5, $T$22:$AB$39, 2, FALSE))</f>
         <v>0.25</v>
       </c>
-      <c r="J5" s="16">
-        <f>IF(ISBLANK($A5), "", VLOOKUP($B5, $T$22:$AB$39, 3, FALSE))</f>
+      <c r="J5" s="14">
+        <f t="shared" ref="J5:J14" si="2">IF(ISBLANK($A5), "", VLOOKUP($B5, $T$22:$AB$39, 3, FALSE))</f>
         <v>0.45</v>
       </c>
-      <c r="K5" s="16">
-        <f>IF(ISBLANK($A5), "", VLOOKUP($B5, $T$22:$AB$39, 4, FALSE))</f>
+      <c r="K5" s="14">
+        <f t="shared" ref="K5:K14" si="3">IF(ISBLANK($A5), "", VLOOKUP($B5, $T$22:$AB$39, 4, FALSE))</f>
         <v>0.2</v>
       </c>
-      <c r="L5" s="16">
-        <f>IF(ISBLANK($A5), "", VLOOKUP($B5, $T$22:$AB$39, 6, FALSE))</f>
+      <c r="L5" s="14">
+        <f t="shared" ref="L5:L14" si="4">IF(ISBLANK($A5), "", VLOOKUP($B5, $T$22:$AB$39, 6, FALSE))</f>
         <v>5.0000000000000001E-3</v>
       </c>
-      <c r="M5" s="16">
+      <c r="M5" s="14">
         <f>IF(L5="n/a",0,L5)</f>
         <v>5.0000000000000001E-3</v>
       </c>
-      <c r="N5" s="16">
-        <f>IF(ISBLANK($A5), "", VLOOKUP($B5, $T$22:$AB$39, 7, FALSE))</f>
+      <c r="N5" s="14">
+        <f t="shared" ref="N5:N14" si="5">IF(ISBLANK($A5), "", VLOOKUP($B5, $T$22:$AB$39, 7, FALSE))</f>
         <v>7.0000000000000001E-3</v>
       </c>
-      <c r="O5" s="16">
+      <c r="O5" s="14">
         <f>IF(N5="n/a",0,N5)</f>
         <v>7.0000000000000001E-3</v>
       </c>
       <c r="P5">
-        <f>IF(ISBLANK(A5),"", (H5*I5*(1 - F5 - G5) * K5*M5)+(H5*I5*J5*K5*O5))</f>
+        <f t="shared" ref="P5:P14" si="6">IF(ISBLANK(A5),"", (H5*I5*(1 - F5 - G5) * K5*M5)+(H5*I5*J5*K5*O5))</f>
         <v>35.75</v>
       </c>
       <c r="Q5">
-        <f>IF(ISBLANK(A5),"",VLOOKUP(A5,$T$14:$U$30,2,FALSE))</f>
+        <f t="shared" ref="Q5:Q14" si="7">IF(ISBLANK(A5),"",VLOOKUP(A5,$T$14:$U$30,2,FALSE))</f>
         <v>6.0000000000000001E-3</v>
       </c>
       <c r="R5">
-        <f>IF(ISBLANK(A5), "", P5*Q5*$U$10/1000)</f>
+        <f t="shared" ref="R5:R14" si="8">IF(ISBLANK(A5), "", P5*Q5*$U$10/1000)</f>
         <v>3.370714285714286E-4</v>
       </c>
     </row>
     <row r="6" spans="1:22">
       <c r="A6" s="2" t="s">
-        <v>53</v>
+        <v>11</v>
       </c>
       <c r="B6" t="s">
-        <v>82</v>
+        <v>40</v>
       </c>
       <c r="C6" t="s">
-        <v>77</v>
+        <v>35</v>
       </c>
       <c r="D6">
         <v>50</v>
@@ -1513,59 +1226,59 @@
         <v>0</v>
       </c>
       <c r="H6">
-        <f>IF(ISBLANK(A6), "", D6*E6)</f>
+        <f t="shared" si="0"/>
         <v>100000</v>
       </c>
-      <c r="I6" s="16">
-        <f>IF(ISBLANK($A6), "", VLOOKUP($B6, $T$22:$AB$39, 2, FALSE))</f>
+      <c r="I6" s="14">
+        <f t="shared" si="1"/>
         <v>0.25</v>
       </c>
-      <c r="J6" s="16">
-        <f>IF(ISBLANK($A6), "", VLOOKUP($B6, $T$22:$AB$39, 3, FALSE))</f>
+      <c r="J6" s="14">
+        <f t="shared" si="2"/>
         <v>0.45</v>
       </c>
-      <c r="K6" s="16">
-        <f>IF(ISBLANK($A6), "", VLOOKUP($B6, $T$22:$AB$39, 4, FALSE))</f>
+      <c r="K6" s="14">
+        <f t="shared" si="3"/>
         <v>0.2</v>
       </c>
-      <c r="L6" s="16">
-        <f>IF(ISBLANK($A6), "", VLOOKUP($B6, $T$22:$AB$39, 6, FALSE))</f>
+      <c r="L6" s="14">
+        <f t="shared" si="4"/>
         <v>5.0000000000000001E-3</v>
       </c>
-      <c r="M6" s="16">
-        <f t="shared" ref="M6:M20" si="0">IF(L6="n/a",0,L6)</f>
+      <c r="M6" s="14">
+        <f t="shared" ref="M6:M20" si="9">IF(L6="n/a",0,L6)</f>
         <v>5.0000000000000001E-3</v>
       </c>
-      <c r="N6" s="16">
-        <f>IF(ISBLANK($A6), "", VLOOKUP($B6, $T$22:$AB$39, 7, FALSE))</f>
+      <c r="N6" s="14">
+        <f t="shared" si="5"/>
         <v>7.0000000000000001E-3</v>
       </c>
       <c r="O6">
-        <f t="shared" ref="O6:O20" si="1">IF(N6="n/a",0,N6)</f>
+        <f t="shared" ref="O6:O20" si="10">IF(N6="n/a",0,N6)</f>
         <v>7.0000000000000001E-3</v>
       </c>
       <c r="P6">
-        <f>IF(ISBLANK(A6),"", (H6*I6*(1 - F6 - G6) * K6*M6)+(H6*I6*J6*K6*O6))</f>
+        <f t="shared" si="6"/>
         <v>35.75</v>
       </c>
       <c r="Q6">
-        <f>IF(ISBLANK(A6),"",VLOOKUP(A6,$T$14:$U$30,2,FALSE))</f>
+        <f t="shared" si="7"/>
         <v>5.0000000000000001E-3</v>
       </c>
       <c r="R6">
-        <f>IF(ISBLANK(A6), "", P6*Q6*$U$10/1000)</f>
+        <f t="shared" si="8"/>
         <v>2.8089285714285711E-4</v>
       </c>
     </row>
     <row r="7" spans="1:22">
       <c r="A7" s="2" t="s">
-        <v>52</v>
+        <v>10</v>
       </c>
       <c r="B7" s="2" t="s">
-        <v>74</v>
+        <v>32</v>
       </c>
       <c r="C7" s="2" t="s">
-        <v>77</v>
+        <v>35</v>
       </c>
       <c r="D7">
         <v>50</v>
@@ -1581,59 +1294,59 @@
         <v>0.06</v>
       </c>
       <c r="H7">
-        <f>IF(ISBLANK(A7), "", D7*E7)</f>
+        <f t="shared" si="0"/>
         <v>100000</v>
       </c>
-      <c r="I7" s="16">
-        <f>IF(ISBLANK($A7), "", VLOOKUP($B7, $T$22:$AB$39, 2, FALSE))</f>
+      <c r="I7" s="14">
+        <f t="shared" si="1"/>
         <v>1.31</v>
       </c>
-      <c r="J7" s="16">
-        <f>IF(ISBLANK($A7), "", VLOOKUP($B7, $T$22:$AB$39, 3, FALSE))</f>
+      <c r="J7" s="14">
+        <f t="shared" si="2"/>
         <v>0.16</v>
       </c>
-      <c r="K7" s="16">
-        <f>IF(ISBLANK($A7), "", VLOOKUP($B7, $T$22:$AB$39, 4, FALSE))</f>
+      <c r="K7" s="14">
+        <f t="shared" si="3"/>
         <v>0.8</v>
       </c>
-      <c r="L7" s="16">
-        <f>IF(ISBLANK($A7), "", VLOOKUP($B7, $T$22:$AB$39, 6, FALSE))</f>
+      <c r="L7" s="14">
+        <f t="shared" si="4"/>
         <v>7.0000000000000001E-3</v>
       </c>
-      <c r="M7" s="16">
-        <f t="shared" si="0"/>
+      <c r="M7" s="14">
+        <f t="shared" si="9"/>
         <v>7.0000000000000001E-3</v>
       </c>
-      <c r="N7" s="16">
-        <f>IF(ISBLANK($A7), "", VLOOKUP($B7, $T$22:$AB$39, 7, FALSE))</f>
+      <c r="N7" s="14">
+        <f t="shared" si="5"/>
         <v>0.01</v>
       </c>
       <c r="O7">
-        <f t="shared" si="1"/>
+        <f t="shared" si="10"/>
         <v>0.01</v>
       </c>
       <c r="P7">
-        <f>IF(ISBLANK(A7),"", (H7*I7*(1 - F7 - G7) * K7*M7)+(H7*I7*J7*K7*O7))</f>
+        <f t="shared" si="6"/>
         <v>710.5440000000001</v>
       </c>
       <c r="Q7">
-        <f>IF(ISBLANK(A7),"",VLOOKUP(A7,$T$14:$U$30,2,FALSE))</f>
+        <f t="shared" si="7"/>
         <v>6.0000000000000001E-3</v>
       </c>
       <c r="R7">
-        <f>IF(ISBLANK(A7), "", P7*Q7*$U$10/1000)</f>
+        <f t="shared" si="8"/>
         <v>6.6994148571428583E-3</v>
       </c>
     </row>
     <row r="8" spans="1:22">
       <c r="A8" s="2" t="s">
-        <v>52</v>
+        <v>10</v>
       </c>
       <c r="B8" s="2" t="s">
-        <v>74</v>
+        <v>32</v>
       </c>
       <c r="C8" s="2" t="s">
-        <v>80</v>
+        <v>38</v>
       </c>
       <c r="D8">
         <v>50</v>
@@ -1649,47 +1362,47 @@
         <v>0.06</v>
       </c>
       <c r="H8">
-        <f>IF(ISBLANK(A8), "", D8*E8)</f>
+        <f t="shared" si="0"/>
         <v>100000</v>
       </c>
-      <c r="I8" s="16">
-        <f>IF(ISBLANK($A8), "", VLOOKUP($B8, $T$22:$AB$39, 2, FALSE))</f>
+      <c r="I8" s="14">
+        <f t="shared" si="1"/>
         <v>1.31</v>
       </c>
-      <c r="J8" s="16">
-        <f>IF(ISBLANK($A8), "", VLOOKUP($B8, $T$22:$AB$39, 3, FALSE))</f>
+      <c r="J8" s="14">
+        <f t="shared" si="2"/>
         <v>0.16</v>
       </c>
-      <c r="K8" s="16">
-        <f>IF(ISBLANK($A8), "", VLOOKUP($B8, $T$22:$AB$39, 4, FALSE))</f>
+      <c r="K8" s="14">
+        <f t="shared" si="3"/>
         <v>0.8</v>
       </c>
-      <c r="L8" s="16">
-        <f>IF(ISBLANK($A8), "", VLOOKUP($B8, $T$22:$AB$39, 6, FALSE))</f>
+      <c r="L8" s="14">
+        <f t="shared" si="4"/>
         <v>7.0000000000000001E-3</v>
       </c>
-      <c r="M8" s="16">
-        <f t="shared" si="0"/>
+      <c r="M8" s="14">
+        <f t="shared" si="9"/>
         <v>7.0000000000000001E-3</v>
       </c>
-      <c r="N8" s="16">
-        <f>IF(ISBLANK($A8), "", VLOOKUP($B8, $T$22:$AB$39, 7, FALSE))</f>
+      <c r="N8" s="14">
+        <f t="shared" si="5"/>
         <v>0.01</v>
       </c>
       <c r="O8">
-        <f t="shared" si="1"/>
+        <f t="shared" si="10"/>
         <v>0.01</v>
       </c>
       <c r="P8">
-        <f>IF(ISBLANK(A8),"", (H8*I8*(1 - F8 - G8) * K8*M8)+(H8*I8*J8*K8*O8))</f>
+        <f t="shared" si="6"/>
         <v>710.5440000000001</v>
       </c>
       <c r="Q8">
-        <f>IF(ISBLANK(A8),"",VLOOKUP(A8,$T$14:$U$30,2,FALSE))</f>
+        <f t="shared" si="7"/>
         <v>6.0000000000000001E-3</v>
       </c>
       <c r="R8">
-        <f>IF(ISBLANK(A8), "", P8*Q8*$U$10/1000)</f>
+        <f t="shared" si="8"/>
         <v>6.6994148571428583E-3</v>
       </c>
       <c r="T8" s="2"/>
@@ -1697,13 +1410,13 @@
     </row>
     <row r="9" spans="1:22">
       <c r="A9" s="2" t="s">
-        <v>52</v>
+        <v>10</v>
       </c>
       <c r="B9" s="2" t="s">
-        <v>106</v>
+        <v>64</v>
       </c>
       <c r="C9" s="2" t="s">
-        <v>78</v>
+        <v>36</v>
       </c>
       <c r="D9">
         <v>50</v>
@@ -1719,47 +1432,47 @@
         <v>1</v>
       </c>
       <c r="H9">
-        <f>IF(ISBLANK(A9), "", D9*E9)</f>
+        <f t="shared" si="0"/>
         <v>100000</v>
       </c>
-      <c r="I9" s="16">
-        <f>IF(ISBLANK($A9), "", VLOOKUP($B9, $T$22:$AB$39, 2, FALSE))</f>
+      <c r="I9" s="14">
+        <f t="shared" si="1"/>
         <v>0.34</v>
       </c>
-      <c r="J9" s="16">
-        <f>IF(ISBLANK($A9), "", VLOOKUP($B9, $T$22:$AB$39, 3, FALSE))</f>
+      <c r="J9" s="14">
+        <f t="shared" si="2"/>
         <v>0.43</v>
       </c>
-      <c r="K9" s="16">
-        <f>IF(ISBLANK($A9), "", VLOOKUP($B9, $T$22:$AB$39, 4, FALSE))</f>
+      <c r="K9" s="14">
+        <f t="shared" si="3"/>
         <v>0.25</v>
       </c>
-      <c r="L9" s="16">
-        <f>IF(ISBLANK($A9), "", VLOOKUP($B9, $T$22:$AB$39, 6, FALSE))</f>
+      <c r="L9" s="14">
+        <f t="shared" si="4"/>
         <v>0.02</v>
       </c>
-      <c r="M9" s="16">
-        <f t="shared" si="0"/>
+      <c r="M9" s="14">
+        <f t="shared" si="9"/>
         <v>0.02</v>
       </c>
-      <c r="N9" s="16">
-        <f>IF(ISBLANK($A9), "", VLOOKUP($B9, $T$22:$AB$39, 7, FALSE))</f>
+      <c r="N9" s="14">
+        <f t="shared" si="5"/>
         <v>0.01</v>
       </c>
       <c r="O9">
-        <f t="shared" si="1"/>
+        <f t="shared" si="10"/>
         <v>0.01</v>
       </c>
       <c r="P9">
-        <f>IF(ISBLANK(A9),"", (H9*I9*(1 - F9 - G9) * K9*M9)+(H9*I9*J9*K9*O9))</f>
+        <f t="shared" si="6"/>
         <v>2.5500000000000114</v>
       </c>
       <c r="Q9">
-        <f>IF(ISBLANK(A9),"",VLOOKUP(A9,$T$14:$U$30,2,FALSE))</f>
+        <f t="shared" si="7"/>
         <v>6.0000000000000001E-3</v>
       </c>
       <c r="R9">
-        <f>IF(ISBLANK(A9), "", P9*Q9*$U$10/1000)</f>
+        <f t="shared" si="8"/>
         <v>2.4042857142857252E-5</v>
       </c>
       <c r="T9" s="2"/>
@@ -1767,13 +1480,13 @@
     </row>
     <row r="10" spans="1:22">
       <c r="A10" s="2" t="s">
-        <v>52</v>
+        <v>10</v>
       </c>
       <c r="B10" s="2" t="s">
-        <v>106</v>
+        <v>64</v>
       </c>
       <c r="C10" s="2" t="s">
-        <v>79</v>
+        <v>37</v>
       </c>
       <c r="D10">
         <v>50</v>
@@ -1789,47 +1502,47 @@
         <v>1</v>
       </c>
       <c r="H10">
-        <f>IF(ISBLANK(A10), "", D10*E10)</f>
+        <f t="shared" si="0"/>
         <v>100000</v>
       </c>
-      <c r="I10" s="16">
-        <f>IF(ISBLANK($A10), "", VLOOKUP($B10, $T$22:$AB$39, 2, FALSE))</f>
+      <c r="I10" s="14">
+        <f t="shared" si="1"/>
         <v>0.34</v>
       </c>
-      <c r="J10" s="16">
-        <f>IF(ISBLANK($A10), "", VLOOKUP($B10, $T$22:$AB$39, 3, FALSE))</f>
+      <c r="J10" s="14">
+        <f t="shared" si="2"/>
         <v>0.43</v>
       </c>
-      <c r="K10" s="16">
-        <f>IF(ISBLANK($A10), "", VLOOKUP($B10, $T$22:$AB$39, 4, FALSE))</f>
+      <c r="K10" s="14">
+        <f t="shared" si="3"/>
         <v>0.25</v>
       </c>
-      <c r="L10" s="16">
-        <f>IF(ISBLANK($A10), "", VLOOKUP($B10, $T$22:$AB$39, 6, FALSE))</f>
+      <c r="L10" s="14">
+        <f t="shared" si="4"/>
         <v>0.02</v>
       </c>
-      <c r="M10" s="16">
-        <f t="shared" si="0"/>
+      <c r="M10" s="14">
+        <f t="shared" si="9"/>
         <v>0.02</v>
       </c>
-      <c r="N10" s="16">
-        <f>IF(ISBLANK($A10), "", VLOOKUP($B10, $T$22:$AB$39, 7, FALSE))</f>
+      <c r="N10" s="14">
+        <f t="shared" si="5"/>
         <v>0.01</v>
       </c>
       <c r="O10">
-        <f t="shared" si="1"/>
+        <f t="shared" si="10"/>
         <v>0.01</v>
       </c>
       <c r="P10">
-        <f>IF(ISBLANK(A10),"", (H10*I10*(1 - F10 - G10) * K10*M10)+(H10*I10*J10*K10*O10))</f>
+        <f t="shared" si="6"/>
         <v>-14.450000000000003</v>
       </c>
       <c r="Q10">
-        <f>IF(ISBLANK(A10),"",VLOOKUP(A10,$T$14:$U$30,2,FALSE))</f>
+        <f t="shared" si="7"/>
         <v>6.0000000000000001E-3</v>
       </c>
       <c r="R10">
-        <f>IF(ISBLANK(A10), "", P10*Q10*$U$10/1000)</f>
+        <f t="shared" si="8"/>
         <v>-1.3624285714285717E-4</v>
       </c>
       <c r="T10" t="s">
@@ -1842,13 +1555,13 @@
     </row>
     <row r="11" spans="1:22">
       <c r="A11" s="2" t="s">
-        <v>52</v>
+        <v>10</v>
       </c>
       <c r="B11" s="2" t="s">
-        <v>11</v>
+        <v>3</v>
       </c>
       <c r="C11" s="2" t="s">
-        <v>101</v>
+        <v>59</v>
       </c>
       <c r="D11">
         <v>50</v>
@@ -1864,47 +1577,47 @@
         <v>0</v>
       </c>
       <c r="H11">
-        <f>IF(ISBLANK(A11), "", D11*E11)</f>
+        <f t="shared" si="0"/>
         <v>100000</v>
       </c>
-      <c r="I11" s="16">
-        <f>IF(ISBLANK($A11), "", VLOOKUP($B11, $T$22:$AB$39, 2, FALSE))</f>
+      <c r="I11" s="14">
+        <f t="shared" si="1"/>
         <v>1.9</v>
       </c>
-      <c r="J11" s="16">
-        <f>IF(ISBLANK($A11), "", VLOOKUP($B11, $T$22:$AB$39, 3, FALSE))</f>
+      <c r="J11" s="14">
+        <f t="shared" si="2"/>
         <v>0.3</v>
       </c>
-      <c r="K11" s="16">
-        <f>IF(ISBLANK($A11), "", VLOOKUP($B11, $T$22:$AB$39, 4, FALSE))</f>
+      <c r="K11" s="14">
+        <f t="shared" si="3"/>
         <v>0.9</v>
       </c>
-      <c r="L11" s="16">
-        <f>IF(ISBLANK($A11), "", VLOOKUP($B11, $T$22:$AB$39, 6, FALSE))</f>
-        <v>0.01</v>
-      </c>
-      <c r="M11" s="16">
-        <f t="shared" si="0"/>
-        <v>0.01</v>
-      </c>
-      <c r="N11" s="16">
-        <f>IF(ISBLANK($A11), "", VLOOKUP($B11, $T$22:$AB$39, 7, FALSE))</f>
+      <c r="L11" s="14">
+        <f t="shared" si="4"/>
+        <v>0.01</v>
+      </c>
+      <c r="M11" s="14">
+        <f t="shared" si="9"/>
+        <v>0.01</v>
+      </c>
+      <c r="N11" s="14">
+        <f t="shared" si="5"/>
         <v>0.01</v>
       </c>
       <c r="O11">
-        <f t="shared" si="1"/>
+        <f t="shared" si="10"/>
         <v>0.01</v>
       </c>
       <c r="P11">
-        <f>IF(ISBLANK(A11),"", (H11*I11*(1 - F11 - G11) * K11*M11)+(H11*I11*J11*K11*O11))</f>
+        <f t="shared" si="6"/>
         <v>1710</v>
       </c>
       <c r="Q11">
-        <f>IF(ISBLANK(A11),"",VLOOKUP(A11,$T$14:$U$30,2,FALSE))</f>
+        <f t="shared" si="7"/>
         <v>6.0000000000000001E-3</v>
       </c>
       <c r="R11">
-        <f>IF(ISBLANK(A11), "", P11*Q11*$U$10/1000)</f>
+        <f t="shared" si="8"/>
         <v>1.6122857142857144E-2</v>
       </c>
       <c r="T11" s="2"/>
@@ -1912,13 +1625,13 @@
     </row>
     <row r="12" spans="1:22">
       <c r="A12" s="2" t="s">
-        <v>52</v>
+        <v>10</v>
       </c>
       <c r="B12" s="2" t="s">
-        <v>96</v>
+        <v>54</v>
       </c>
       <c r="C12" s="2" t="s">
-        <v>80</v>
+        <v>38</v>
       </c>
       <c r="D12">
         <v>50</v>
@@ -1934,63 +1647,63 @@
         <v>0</v>
       </c>
       <c r="H12">
-        <f>IF(ISBLANK(A12), "", D12*E12)</f>
+        <f t="shared" si="0"/>
         <v>100000</v>
       </c>
-      <c r="I12" s="16">
-        <f>IF(ISBLANK($A12), "", VLOOKUP($B12, $T$22:$AB$39, 2, FALSE))</f>
+      <c r="I12" s="14">
+        <f t="shared" si="1"/>
         <v>1.5</v>
       </c>
-      <c r="J12" s="16">
-        <f>IF(ISBLANK($A12), "", VLOOKUP($B12, $T$22:$AB$39, 3, FALSE))</f>
+      <c r="J12" s="14">
+        <f t="shared" si="2"/>
         <v>0.28999999999999998</v>
       </c>
-      <c r="K12" s="16">
-        <f>IF(ISBLANK($A12), "", VLOOKUP($B12, $T$22:$AB$39, 4, FALSE))</f>
+      <c r="K12" s="14">
+        <f t="shared" si="3"/>
         <v>0.88</v>
       </c>
-      <c r="L12" s="16">
-        <f>IF(ISBLANK($A12), "", VLOOKUP($B12, $T$22:$AB$39, 6, FALSE))</f>
+      <c r="L12" s="14">
+        <f t="shared" si="4"/>
         <v>6.0000000000000001E-3</v>
       </c>
-      <c r="M12" s="16">
-        <f t="shared" si="0"/>
+      <c r="M12" s="14">
+        <f t="shared" si="9"/>
         <v>6.0000000000000001E-3</v>
       </c>
-      <c r="N12" s="16" t="str">
-        <f>IF(ISBLANK($A12), "", VLOOKUP($B12, $T$22:$AB$39, 7, FALSE))</f>
+      <c r="N12" s="14" t="str">
+        <f t="shared" si="5"/>
         <v>n/a</v>
       </c>
       <c r="O12">
-        <f t="shared" si="1"/>
+        <f t="shared" si="10"/>
         <v>0</v>
       </c>
       <c r="P12">
-        <f>IF(ISBLANK(A12),"", (H12*I12*(1 - F12 - G12) * K12*M12)+(H12*I12*J12*K12*O12))</f>
+        <f t="shared" si="6"/>
         <v>554.4</v>
       </c>
       <c r="Q12">
-        <f>IF(ISBLANK(A12),"",VLOOKUP(A12,$T$14:$U$30,2,FALSE))</f>
+        <f t="shared" si="7"/>
         <v>6.0000000000000001E-3</v>
       </c>
       <c r="R12">
-        <f>IF(ISBLANK(A12), "", P12*Q12*$U$10/1000)</f>
+        <f t="shared" si="8"/>
         <v>5.2271999999999996E-3</v>
       </c>
       <c r="T12" s="2" t="s">
-        <v>48</v>
+        <v>6</v>
       </c>
       <c r="U12" s="2"/>
     </row>
     <row r="13" spans="1:22">
       <c r="A13" s="2" t="s">
-        <v>52</v>
+        <v>10</v>
       </c>
       <c r="B13" s="2" t="s">
-        <v>107</v>
+        <v>65</v>
       </c>
       <c r="C13" s="2" t="s">
-        <v>78</v>
+        <v>36</v>
       </c>
       <c r="D13">
         <v>50</v>
@@ -2006,62 +1719,62 @@
         <v>0.8</v>
       </c>
       <c r="H13">
-        <f>IF(ISBLANK(A13), "", D13*E13)</f>
+        <f t="shared" si="0"/>
         <v>100000</v>
       </c>
-      <c r="I13" s="16">
-        <f>IF(ISBLANK($A13), "", VLOOKUP($B13, $T$22:$AB$39, 2, FALSE))</f>
+      <c r="I13" s="14">
+        <f t="shared" si="1"/>
         <v>1.34</v>
       </c>
-      <c r="J13" s="16">
-        <f>IF(ISBLANK($A13), "", VLOOKUP($B13, $T$22:$AB$39, 3, FALSE))</f>
+      <c r="J13" s="14">
+        <f t="shared" si="2"/>
         <v>0.37</v>
       </c>
-      <c r="K13" s="16">
-        <f>IF(ISBLANK($A13), "", VLOOKUP($B13, $T$22:$AB$39, 4, FALSE))</f>
+      <c r="K13" s="14">
+        <f t="shared" si="3"/>
         <v>0.88</v>
       </c>
-      <c r="L13" s="16">
-        <f>IF(ISBLANK($A13), "", VLOOKUP($B13, $T$22:$AB$39, 6, FALSE))</f>
+      <c r="L13" s="14">
+        <f t="shared" si="4"/>
         <v>6.0000000000000001E-3</v>
       </c>
-      <c r="M13" s="16">
-        <f t="shared" si="0"/>
+      <c r="M13" s="14">
+        <f t="shared" si="9"/>
         <v>6.0000000000000001E-3</v>
       </c>
-      <c r="N13" s="16">
-        <f>IF(ISBLANK($A13), "", VLOOKUP($B13, $T$22:$AB$39, 7, FALSE))</f>
+      <c r="N13" s="14">
+        <f t="shared" si="5"/>
         <v>0.01</v>
       </c>
       <c r="O13">
-        <f t="shared" si="1"/>
+        <f t="shared" si="10"/>
         <v>0.01</v>
       </c>
       <c r="P13">
-        <f>IF(ISBLANK(A13),"", (H13*I13*(1 - F13 - G13) * K13*M13)+(H13*I13*J13*K13*O13))</f>
+        <f t="shared" si="6"/>
         <v>365.55199999999996</v>
       </c>
       <c r="Q13">
-        <f>IF(ISBLANK(A13),"",VLOOKUP(A13,$T$14:$U$30,2,FALSE))</f>
+        <f t="shared" si="7"/>
         <v>6.0000000000000001E-3</v>
       </c>
       <c r="R13">
-        <f>IF(ISBLANK(A13), "", P13*Q13*$U$10/1000)</f>
+        <f t="shared" si="8"/>
         <v>3.4466331428571425E-3</v>
       </c>
       <c r="T13" t="s">
-        <v>49</v>
+        <v>7</v>
       </c>
     </row>
     <row r="14" spans="1:22">
       <c r="A14" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="B14" s="2" t="s">
         <v>52</v>
       </c>
-      <c r="B14" s="2" t="s">
-        <v>94</v>
-      </c>
-      <c r="C14" s="15" t="s">
-        <v>80</v>
+      <c r="C14" s="13" t="s">
+        <v>38</v>
       </c>
       <c r="D14">
         <v>50</v>
@@ -2077,105 +1790,105 @@
         <v>7.0000000000000007E-2</v>
       </c>
       <c r="H14">
-        <f>IF(ISBLANK(A14), "", D14*E14)</f>
+        <f t="shared" si="0"/>
         <v>100000</v>
       </c>
-      <c r="I14" s="16">
-        <f>IF(ISBLANK($A14), "", VLOOKUP($B14, $T$22:$AB$39, 2, FALSE))</f>
+      <c r="I14" s="14">
+        <f t="shared" si="1"/>
         <v>1.37</v>
       </c>
-      <c r="J14" s="16">
-        <f>IF(ISBLANK($A14), "", VLOOKUP($B14, $T$22:$AB$39, 3, FALSE))</f>
+      <c r="J14" s="14">
+        <f t="shared" si="2"/>
         <v>0.51</v>
       </c>
-      <c r="K14" s="16">
-        <f>IF(ISBLANK($A14), "", VLOOKUP($B14, $T$22:$AB$39, 4, FALSE))</f>
+      <c r="K14" s="14">
+        <f t="shared" si="3"/>
         <v>0.87</v>
       </c>
-      <c r="L14" s="16">
-        <f>IF(ISBLANK($A14), "", VLOOKUP($B14, $T$22:$AB$39, 6, FALSE))</f>
+      <c r="L14" s="14">
+        <f t="shared" si="4"/>
         <v>8.9999999999999993E-3</v>
       </c>
-      <c r="M14" s="16">
-        <f t="shared" si="0"/>
+      <c r="M14" s="14">
+        <f t="shared" si="9"/>
         <v>8.9999999999999993E-3</v>
       </c>
-      <c r="N14" s="16">
-        <f>IF(ISBLANK($A14), "", VLOOKUP($B14, $T$22:$AB$39, 7, FALSE))</f>
+      <c r="N14" s="14">
+        <f t="shared" si="5"/>
         <v>0.01</v>
       </c>
       <c r="O14">
-        <f t="shared" si="1"/>
+        <f t="shared" si="10"/>
         <v>0.01</v>
       </c>
       <c r="P14">
-        <f>IF(ISBLANK(A14),"", (H14*I14*(1 - F14 - G14) * K14*M14)+(H14*I14*J14*K14*O14))</f>
+        <f t="shared" si="6"/>
         <v>1283.6762999999999</v>
       </c>
       <c r="Q14">
-        <f>IF(ISBLANK(A14),"",VLOOKUP(A14,$T$14:$U$30,2,FALSE))</f>
+        <f t="shared" si="7"/>
         <v>6.0000000000000001E-3</v>
       </c>
       <c r="R14">
-        <f>IF(ISBLANK(A14), "", P14*Q14*$U$10/1000)</f>
+        <f t="shared" si="8"/>
         <v>1.2103233685714285E-2</v>
       </c>
       <c r="T14" s="2" t="s">
-        <v>52</v>
+        <v>10</v>
       </c>
       <c r="U14" s="2">
         <v>6.0000000000000001E-3</v>
       </c>
-      <c r="V14" s="11" t="s">
-        <v>50</v>
+      <c r="V14" s="9" t="s">
+        <v>8</v>
       </c>
     </row>
     <row r="15" spans="1:22">
       <c r="A15" s="2"/>
       <c r="B15" s="2"/>
-      <c r="C15" s="15"/>
-      <c r="I15" s="16"/>
-      <c r="J15" s="16"/>
-      <c r="K15" s="16"/>
-      <c r="L15" s="16"/>
-      <c r="M15" s="16"/>
-      <c r="N15" s="16"/>
+      <c r="C15" s="13"/>
+      <c r="I15" s="14"/>
+      <c r="J15" s="14"/>
+      <c r="K15" s="14"/>
+      <c r="L15" s="14"/>
+      <c r="M15" s="14"/>
+      <c r="N15" s="14"/>
       <c r="T15" s="2" t="s">
-        <v>53</v>
+        <v>11</v>
       </c>
       <c r="U15" s="2">
         <v>5.0000000000000001E-3</v>
       </c>
-      <c r="V15" s="11" t="s">
-        <v>51</v>
+      <c r="V15" s="9" t="s">
+        <v>9</v>
       </c>
     </row>
     <row r="16" spans="1:22">
       <c r="A16" s="2"/>
       <c r="B16" s="2"/>
-      <c r="C16" s="15"/>
+      <c r="C16" s="13"/>
       <c r="G16" s="5" t="s">
-        <v>114</v>
-      </c>
-      <c r="I16" s="16"/>
-      <c r="J16" s="16"/>
-      <c r="K16" s="16"/>
-      <c r="L16" s="16"/>
-      <c r="M16" s="16"/>
-      <c r="N16" s="16"/>
+        <v>72</v>
+      </c>
+      <c r="I16" s="14"/>
+      <c r="J16" s="14"/>
+      <c r="K16" s="14"/>
+      <c r="L16" s="14"/>
+      <c r="M16" s="14"/>
+      <c r="N16" s="14"/>
       <c r="T16" s="2"/>
       <c r="U16" s="2"/>
-      <c r="V16" s="11"/>
+      <c r="V16" s="9"/>
     </row>
     <row r="17" spans="1:28">
       <c r="A17" s="2" t="s">
-        <v>52</v>
+        <v>10</v>
       </c>
       <c r="B17" s="2" t="s">
-        <v>74</v>
-      </c>
-      <c r="C17" s="15" t="s">
-        <v>104</v>
+        <v>32</v>
+      </c>
+      <c r="C17" s="13" t="s">
+        <v>62</v>
       </c>
       <c r="D17">
         <v>50</v>
@@ -2193,32 +1906,32 @@
         <f>IF(ISBLANK(A17), "", D17*E17)</f>
         <v>100000</v>
       </c>
-      <c r="I17" s="16">
+      <c r="I17" s="14">
         <f>IF(ISBLANK($A17), "", VLOOKUP($B17, $T$22:$AB$39, 2, FALSE))</f>
         <v>1.31</v>
       </c>
-      <c r="J17" s="16">
+      <c r="J17" s="14">
         <f>IF(ISBLANK($A17), "", VLOOKUP($B17, $T$22:$AB$39, 3, FALSE))</f>
         <v>0.16</v>
       </c>
-      <c r="K17" s="16">
+      <c r="K17" s="14">
         <f>IF(ISBLANK($A17), "", VLOOKUP($B17, $T$22:$AB$39, 4, FALSE))</f>
         <v>0.8</v>
       </c>
-      <c r="L17" s="16">
+      <c r="L17" s="14">
         <f>IF(ISBLANK($A17), "", VLOOKUP($B17, $T$22:$AB$39, 6, FALSE))</f>
         <v>7.0000000000000001E-3</v>
       </c>
-      <c r="M17" s="16">
-        <f t="shared" si="0"/>
+      <c r="M17" s="14">
+        <f t="shared" si="9"/>
         <v>7.0000000000000001E-3</v>
       </c>
-      <c r="N17" s="16">
+      <c r="N17" s="14">
         <f>IF(ISBLANK($A17), "", VLOOKUP($B17, $T$22:$AB$39, 7, FALSE))</f>
         <v>0.01</v>
       </c>
       <c r="O17">
-        <f t="shared" si="1"/>
+        <f t="shared" si="10"/>
         <v>0.01</v>
       </c>
       <c r="P17">
@@ -2236,13 +1949,13 @@
     </row>
     <row r="18" spans="1:28">
       <c r="A18" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="B18" s="2" t="s">
         <v>52</v>
       </c>
-      <c r="B18" s="2" t="s">
-        <v>94</v>
-      </c>
-      <c r="C18" s="15" t="s">
-        <v>80</v>
+      <c r="C18" s="13" t="s">
+        <v>38</v>
       </c>
       <c r="D18">
         <v>50</v>
@@ -2260,32 +1973,32 @@
         <f>IF(ISBLANK(A18), "", D18*E18)</f>
         <v>100000</v>
       </c>
-      <c r="I18" s="16">
+      <c r="I18" s="14">
         <f>IF(ISBLANK($A18), "", VLOOKUP($B18, $T$22:$AB$39, 2, FALSE))</f>
         <v>1.37</v>
       </c>
-      <c r="J18" s="16">
+      <c r="J18" s="14">
         <f>IF(ISBLANK($A18), "", VLOOKUP($B18, $T$22:$AB$39, 3, FALSE))</f>
         <v>0.51</v>
       </c>
-      <c r="K18" s="16">
+      <c r="K18" s="14">
         <f>IF(ISBLANK($A18), "", VLOOKUP($B18, $T$22:$AB$39, 4, FALSE))</f>
         <v>0.87</v>
       </c>
-      <c r="L18" s="16">
+      <c r="L18" s="14">
         <f>IF(ISBLANK($A18), "", VLOOKUP($B18, $T$22:$AB$39, 6, FALSE))</f>
         <v>8.9999999999999993E-3</v>
       </c>
-      <c r="M18" s="16">
-        <f t="shared" si="0"/>
+      <c r="M18" s="14">
+        <f t="shared" si="9"/>
         <v>8.9999999999999993E-3</v>
       </c>
-      <c r="N18" s="16">
+      <c r="N18" s="14">
         <f>IF(ISBLANK($A18), "", VLOOKUP($B18, $T$22:$AB$39, 7, FALSE))</f>
         <v>0.01</v>
       </c>
       <c r="O18">
-        <f t="shared" si="1"/>
+        <f t="shared" si="10"/>
         <v>0.01</v>
       </c>
       <c r="P18">
@@ -2305,13 +2018,13 @@
     </row>
     <row r="19" spans="1:28">
       <c r="A19" s="2" t="s">
-        <v>52</v>
+        <v>10</v>
       </c>
       <c r="B19" s="2" t="s">
-        <v>96</v>
-      </c>
-      <c r="C19" s="15" t="s">
-        <v>80</v>
+        <v>54</v>
+      </c>
+      <c r="C19" s="13" t="s">
+        <v>38</v>
       </c>
       <c r="D19">
         <v>50</v>
@@ -2329,32 +2042,32 @@
         <f>IF(ISBLANK(A19), "", D19*E19)</f>
         <v>100000</v>
       </c>
-      <c r="I19" s="16">
+      <c r="I19" s="14">
         <f>IF(ISBLANK($A19), "", VLOOKUP($B19, $T$22:$AB$39, 2, FALSE))</f>
         <v>1.5</v>
       </c>
-      <c r="J19" s="16">
+      <c r="J19" s="14">
         <f>IF(ISBLANK($A19), "", VLOOKUP($B19, $T$22:$AB$39, 3, FALSE))</f>
         <v>0.28999999999999998</v>
       </c>
-      <c r="K19" s="16">
+      <c r="K19" s="14">
         <f>IF(ISBLANK($A19), "", VLOOKUP($B19, $T$22:$AB$39, 4, FALSE))</f>
         <v>0.88</v>
       </c>
-      <c r="L19" s="16">
+      <c r="L19" s="14">
         <f>IF(ISBLANK($A19), "", VLOOKUP($B19, $T$22:$AB$39, 6, FALSE))</f>
         <v>6.0000000000000001E-3</v>
       </c>
-      <c r="M19" s="16">
-        <f t="shared" si="0"/>
+      <c r="M19" s="14">
+        <f t="shared" si="9"/>
         <v>6.0000000000000001E-3</v>
       </c>
-      <c r="N19" s="16" t="str">
+      <c r="N19" s="14" t="str">
         <f>IF(ISBLANK($A19), "", VLOOKUP($B19, $T$22:$AB$39, 7, FALSE))</f>
         <v>n/a</v>
       </c>
       <c r="O19">
-        <f t="shared" si="1"/>
+        <f t="shared" si="10"/>
         <v>0</v>
       </c>
       <c r="P19">
@@ -2374,13 +2087,13 @@
     </row>
     <row r="20" spans="1:28">
       <c r="A20" s="2" t="s">
-        <v>52</v>
+        <v>10</v>
       </c>
       <c r="B20" s="2" t="s">
-        <v>113</v>
-      </c>
-      <c r="C20" s="15" t="s">
-        <v>77</v>
+        <v>71</v>
+      </c>
+      <c r="C20" s="13" t="s">
+        <v>35</v>
       </c>
       <c r="D20">
         <v>50</v>
@@ -2398,32 +2111,32 @@
         <f>IF(ISBLANK(A20), "", D20*E20)</f>
         <v>100000</v>
       </c>
-      <c r="I20" s="16">
+      <c r="I20" s="14">
         <f>IF(ISBLANK($A20), "", VLOOKUP($B20, $T$22:$AB$39, 2, FALSE))</f>
         <v>1</v>
       </c>
-      <c r="J20" s="16">
+      <c r="J20" s="14">
         <f>IF(ISBLANK($A20), "", VLOOKUP($B20, $T$22:$AB$39, 3, FALSE))</f>
         <v>0.22</v>
       </c>
-      <c r="K20" s="16">
+      <c r="K20" s="14">
         <f>IF(ISBLANK($A20), "", VLOOKUP($B20, $T$22:$AB$39, 4, FALSE))</f>
         <v>0.85</v>
       </c>
-      <c r="L20" s="16">
+      <c r="L20" s="14">
         <f>IF(ISBLANK($A20), "", VLOOKUP($B20, $T$22:$AB$39, 6, FALSE))</f>
         <v>8.0000000000000002E-3</v>
       </c>
-      <c r="M20" s="16">
-        <f t="shared" si="0"/>
+      <c r="M20" s="14">
+        <f t="shared" si="9"/>
         <v>8.0000000000000002E-3</v>
       </c>
-      <c r="N20" s="16">
+      <c r="N20" s="14">
         <f>IF(ISBLANK($A20), "", VLOOKUP($B20, $T$22:$AB$39, 7, FALSE))</f>
         <v>8.9999999999999993E-3</v>
       </c>
       <c r="O20">
-        <f t="shared" si="1"/>
+        <f t="shared" si="10"/>
         <v>8.9999999999999993E-3</v>
       </c>
       <c r="P20">
@@ -2439,95 +2152,95 @@
         <v>-3.3660000000000043E-4</v>
       </c>
       <c r="T20" s="2" t="s">
-        <v>58</v>
+        <v>16</v>
       </c>
       <c r="U20" s="2"/>
     </row>
     <row r="21" spans="1:28" ht="17">
       <c r="T21" s="2"/>
       <c r="U21" s="2" t="s">
-        <v>60</v>
+        <v>18</v>
       </c>
       <c r="V21" t="s">
-        <v>61</v>
+        <v>19</v>
       </c>
       <c r="W21" t="s">
-        <v>62</v>
-      </c>
-      <c r="X21" s="10" t="s">
-        <v>63</v>
+        <v>20</v>
+      </c>
+      <c r="X21" s="8" t="s">
+        <v>21</v>
       </c>
       <c r="Y21" t="s">
-        <v>64</v>
+        <v>22</v>
       </c>
       <c r="Z21" t="s">
-        <v>65</v>
+        <v>23</v>
       </c>
       <c r="AA21" t="s">
-        <v>66</v>
+        <v>24</v>
       </c>
       <c r="AB21" t="s">
-        <v>67</v>
+        <v>25</v>
       </c>
     </row>
     <row r="22" spans="1:28">
       <c r="T22" s="2" t="s">
-        <v>87</v>
-      </c>
-      <c r="U22" s="14">
+        <v>45</v>
+      </c>
+      <c r="U22" s="12">
         <v>1.5</v>
       </c>
-      <c r="V22" s="13">
+      <c r="V22" s="11">
         <v>0.28999999999999998</v>
       </c>
-      <c r="W22" s="13">
+      <c r="W22" s="11">
         <v>0.88</v>
       </c>
-      <c r="X22" s="13">
+      <c r="X22" s="11">
         <v>0.4</v>
       </c>
-      <c r="Y22" s="13">
+      <c r="Y22" s="11">
         <v>6.0000000000000001E-3</v>
       </c>
-      <c r="Z22" s="13">
-        <v>0.01</v>
-      </c>
-      <c r="AA22" s="13">
+      <c r="Z22" s="11">
+        <v>0.01</v>
+      </c>
+      <c r="AA22" s="11">
         <v>0.5</v>
       </c>
-      <c r="AB22" s="13">
+      <c r="AB22" s="11">
         <v>0.9</v>
       </c>
     </row>
     <row r="23" spans="1:28">
       <c r="B23" s="2"/>
       <c r="C23" s="2"/>
-      <c r="N23" s="16"/>
+      <c r="N23" s="14"/>
       <c r="T23" s="2" t="s">
-        <v>88</v>
-      </c>
-      <c r="U23" s="14">
+        <v>46</v>
+      </c>
+      <c r="U23" s="12">
         <v>1.24</v>
       </c>
-      <c r="V23" s="13">
+      <c r="V23" s="11">
         <v>0.32</v>
       </c>
-      <c r="W23" s="13">
+      <c r="W23" s="11">
         <v>0.88</v>
       </c>
-      <c r="X23" s="13">
+      <c r="X23" s="11">
         <v>0.4</v>
       </c>
-      <c r="Y23" s="13">
+      <c r="Y23" s="11">
         <v>7.0000000000000001E-3</v>
       </c>
-      <c r="Z23" s="13">
-        <v>0.01</v>
-      </c>
-      <c r="AA23" s="13">
+      <c r="Z23" s="11">
+        <v>0.01</v>
+      </c>
+      <c r="AA23" s="11">
         <v>0.5</v>
       </c>
-      <c r="AB23" s="13">
+      <c r="AB23" s="11">
         <v>0.85</v>
       </c>
     </row>
@@ -2535,30 +2248,30 @@
       <c r="B24" s="2"/>
       <c r="C24" s="2"/>
       <c r="T24" s="2" t="s">
-        <v>89</v>
-      </c>
-      <c r="U24" s="14">
+        <v>47</v>
+      </c>
+      <c r="U24" s="12">
         <v>0.81</v>
       </c>
-      <c r="V24" s="13">
+      <c r="V24" s="11">
         <v>0.39</v>
       </c>
-      <c r="W24" s="13">
+      <c r="W24" s="11">
         <v>0.85</v>
       </c>
-      <c r="X24" s="13">
+      <c r="X24" s="11">
         <v>0.42</v>
       </c>
-      <c r="Y24" s="13">
+      <c r="Y24" s="11">
         <v>5.0000000000000001E-3</v>
       </c>
-      <c r="Z24" s="13">
+      <c r="Z24" s="11">
         <v>7.0000000000000001E-3</v>
       </c>
-      <c r="AA24" s="13">
+      <c r="AA24" s="11">
         <v>1</v>
       </c>
-      <c r="AB24" s="13">
+      <c r="AB24" s="11">
         <v>0.8</v>
       </c>
     </row>
@@ -2568,30 +2281,30 @@
         <v/>
       </c>
       <c r="T25" s="2" t="s">
-        <v>90</v>
-      </c>
-      <c r="U25" s="14">
+        <v>48</v>
+      </c>
+      <c r="U25" s="12">
         <v>1.42</v>
       </c>
-      <c r="V25" s="13">
+      <c r="V25" s="11">
         <v>0.43</v>
       </c>
-      <c r="W25" s="13">
+      <c r="W25" s="11">
         <v>0.88</v>
       </c>
-      <c r="X25" s="13">
+      <c r="X25" s="11">
         <v>0.4</v>
       </c>
-      <c r="Y25" s="13">
+      <c r="Y25" s="11">
         <v>6.0000000000000001E-3</v>
       </c>
-      <c r="Z25" s="13">
-        <v>0.01</v>
-      </c>
-      <c r="AA25" s="13">
+      <c r="Z25" s="11">
+        <v>0.01</v>
+      </c>
+      <c r="AA25" s="11">
         <v>0.5</v>
       </c>
-      <c r="AB25" s="13">
+      <c r="AB25" s="11">
         <v>0.85</v>
       </c>
     </row>
@@ -2601,30 +2314,30 @@
         <v/>
       </c>
       <c r="T26" s="2" t="s">
-        <v>74</v>
-      </c>
-      <c r="U26" s="14">
+        <v>32</v>
+      </c>
+      <c r="U26" s="12">
         <v>1.31</v>
       </c>
-      <c r="V26" s="13">
+      <c r="V26" s="11">
         <v>0.16</v>
       </c>
-      <c r="W26" s="13">
+      <c r="W26" s="11">
         <v>0.8</v>
       </c>
-      <c r="X26" s="13">
+      <c r="X26" s="11">
         <v>0.42</v>
       </c>
-      <c r="Y26" s="13">
+      <c r="Y26" s="11">
         <v>7.0000000000000001E-3</v>
       </c>
-      <c r="Z26" s="13">
-        <v>0.01</v>
-      </c>
-      <c r="AA26" s="13">
+      <c r="Z26" s="11">
+        <v>0.01</v>
+      </c>
+      <c r="AA26" s="11">
         <v>1</v>
       </c>
-      <c r="AB26" s="13">
+      <c r="AB26" s="11">
         <v>0.8</v>
       </c>
     </row>
@@ -2634,30 +2347,30 @@
         <v/>
       </c>
       <c r="T27" s="2" t="s">
-        <v>91</v>
-      </c>
-      <c r="U27" s="14">
+        <v>49</v>
+      </c>
+      <c r="U27" s="12">
         <v>1.5</v>
       </c>
-      <c r="V27" s="13">
+      <c r="V27" s="11">
         <v>0.22</v>
       </c>
-      <c r="W27" s="13">
+      <c r="W27" s="11">
         <v>0.8</v>
       </c>
-      <c r="X27" s="13">
+      <c r="X27" s="11">
         <v>0.4</v>
       </c>
-      <c r="Y27" s="13">
+      <c r="Y27" s="11">
         <v>8.0000000000000002E-3</v>
       </c>
-      <c r="Z27" s="13">
+      <c r="Z27" s="11">
         <v>7.0000000000000001E-3</v>
       </c>
-      <c r="AA27" s="13">
+      <c r="AA27" s="11">
         <v>0.5</v>
       </c>
-      <c r="AB27" s="13">
+      <c r="AB27" s="11">
         <v>0.85</v>
       </c>
     </row>
@@ -2667,362 +2380,362 @@
         <v/>
       </c>
       <c r="T28" s="2" t="s">
-        <v>92</v>
-      </c>
-      <c r="U28" s="14">
+        <v>50</v>
+      </c>
+      <c r="U28" s="12">
         <v>1.5</v>
       </c>
-      <c r="V28" s="13">
+      <c r="V28" s="11">
         <v>0.42</v>
       </c>
-      <c r="W28" s="13">
+      <c r="W28" s="11">
         <v>0.88</v>
       </c>
-      <c r="X28" s="13">
+      <c r="X28" s="11">
         <v>0.4</v>
       </c>
-      <c r="Y28" s="13">
+      <c r="Y28" s="11">
         <v>6.0000000000000001E-3</v>
       </c>
-      <c r="Z28" s="13">
-        <v>0.01</v>
-      </c>
-      <c r="AA28" s="13">
+      <c r="Z28" s="11">
+        <v>0.01</v>
+      </c>
+      <c r="AA28" s="11">
         <v>0.5</v>
       </c>
-      <c r="AB28" s="13">
+      <c r="AB28" s="11">
         <v>0.85</v>
       </c>
     </row>
     <row r="29" spans="1:28">
       <c r="T29" s="2" t="s">
-        <v>93</v>
-      </c>
-      <c r="U29" s="14">
+        <v>51</v>
+      </c>
+      <c r="U29" s="12">
         <v>1.46</v>
       </c>
-      <c r="V29" s="13">
+      <c r="V29" s="11">
         <v>0.36</v>
       </c>
-      <c r="W29" s="13">
+      <c r="W29" s="11">
         <v>0.88</v>
       </c>
-      <c r="X29" s="13">
+      <c r="X29" s="11">
         <v>0.4</v>
       </c>
-      <c r="Y29" s="13">
+      <c r="Y29" s="11">
         <v>6.0000000000000001E-3</v>
       </c>
-      <c r="Z29" s="13">
-        <v>0.01</v>
-      </c>
-      <c r="AA29" s="13">
+      <c r="Z29" s="11">
+        <v>0.01</v>
+      </c>
+      <c r="AA29" s="11">
         <v>0.5</v>
       </c>
-      <c r="AB29" s="13">
+      <c r="AB29" s="11">
         <v>0.85</v>
       </c>
     </row>
     <row r="30" spans="1:28">
       <c r="T30" s="2" t="s">
-        <v>94</v>
-      </c>
-      <c r="U30" s="14">
+        <v>52</v>
+      </c>
+      <c r="U30" s="12">
         <v>1.37</v>
       </c>
-      <c r="V30" s="13">
+      <c r="V30" s="11">
         <v>0.51</v>
       </c>
-      <c r="W30" s="13">
+      <c r="W30" s="11">
         <v>0.87</v>
       </c>
-      <c r="X30" s="13">
+      <c r="X30" s="11">
         <v>0.4</v>
       </c>
-      <c r="Y30" s="13">
+      <c r="Y30" s="11">
         <v>8.9999999999999993E-3</v>
       </c>
-      <c r="Z30" s="13">
-        <v>0.01</v>
-      </c>
-      <c r="AA30" s="13">
+      <c r="Z30" s="11">
+        <v>0.01</v>
+      </c>
+      <c r="AA30" s="11">
         <v>0.5</v>
       </c>
-      <c r="AB30" s="13">
+      <c r="AB30" s="11">
         <v>0.85</v>
       </c>
     </row>
     <row r="31" spans="1:28">
       <c r="T31" s="2" t="s">
-        <v>76</v>
-      </c>
-      <c r="U31" s="14">
+        <v>34</v>
+      </c>
+      <c r="U31" s="12">
         <v>0.34</v>
       </c>
-      <c r="V31" s="13">
+      <c r="V31" s="11">
         <v>0.43</v>
       </c>
-      <c r="W31" s="13">
+      <c r="W31" s="11">
         <v>0.25</v>
       </c>
-      <c r="X31" s="13">
+      <c r="X31" s="11">
         <v>0.4</v>
       </c>
-      <c r="Y31" s="13">
+      <c r="Y31" s="11">
         <v>0.02</v>
       </c>
-      <c r="Z31" s="13">
-        <v>0.01</v>
-      </c>
-      <c r="AA31" s="13" t="s">
-        <v>99</v>
-      </c>
-      <c r="AB31" s="13">
+      <c r="Z31" s="11">
+        <v>0.01</v>
+      </c>
+      <c r="AA31" s="11" t="s">
+        <v>57</v>
+      </c>
+      <c r="AB31" s="11">
         <v>0.85</v>
       </c>
     </row>
     <row r="32" spans="1:28">
       <c r="T32" s="2" t="s">
-        <v>95</v>
-      </c>
-      <c r="U32" s="14">
+        <v>53</v>
+      </c>
+      <c r="U32" s="12">
         <v>1.07</v>
       </c>
-      <c r="V32" s="13">
+      <c r="V32" s="11">
         <v>0.2</v>
       </c>
-      <c r="W32" s="13">
+      <c r="W32" s="11">
         <v>0.8</v>
       </c>
-      <c r="X32" s="13">
+      <c r="X32" s="11">
         <v>0.42</v>
       </c>
-      <c r="Y32" s="13">
+      <c r="Y32" s="11">
         <v>1.6E-2</v>
       </c>
-      <c r="Z32" s="13">
+      <c r="Z32" s="11">
         <v>1.4E-2</v>
       </c>
-      <c r="AA32" s="13">
+      <c r="AA32" s="11">
         <v>0.5</v>
       </c>
-      <c r="AB32" s="13">
+      <c r="AB32" s="11">
         <v>0.85</v>
       </c>
     </row>
     <row r="33" spans="20:28">
       <c r="T33" s="2" t="s">
-        <v>86</v>
-      </c>
-      <c r="U33" s="14">
+        <v>44</v>
+      </c>
+      <c r="U33" s="12">
         <v>0.25</v>
       </c>
-      <c r="V33" s="13">
+      <c r="V33" s="11">
         <v>0.45</v>
       </c>
-      <c r="W33" s="13">
+      <c r="W33" s="11">
         <v>0.2</v>
       </c>
-      <c r="X33" s="13">
+      <c r="X33" s="11">
         <v>0.4</v>
       </c>
-      <c r="Y33" s="13">
+      <c r="Y33" s="11">
         <v>5.0000000000000001E-3</v>
       </c>
-      <c r="Z33" s="13">
+      <c r="Z33" s="11">
         <v>7.0000000000000001E-3</v>
       </c>
-      <c r="AA33" s="13">
+      <c r="AA33" s="11">
         <v>1</v>
       </c>
-      <c r="AB33" s="13">
+      <c r="AB33" s="11">
         <v>0.8</v>
       </c>
     </row>
     <row r="34" spans="20:28">
       <c r="T34" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="U34" s="14">
+        <v>3</v>
+      </c>
+      <c r="U34" s="12">
         <v>1.9</v>
       </c>
-      <c r="V34" s="13">
+      <c r="V34" s="11">
         <v>0.3</v>
       </c>
-      <c r="W34" s="13">
+      <c r="W34" s="11">
         <v>0.9</v>
       </c>
-      <c r="X34" s="13">
+      <c r="X34" s="11">
         <v>0.4</v>
       </c>
-      <c r="Y34" s="13">
-        <v>0.01</v>
-      </c>
-      <c r="Z34" s="13">
-        <v>0.01</v>
-      </c>
-      <c r="AA34" s="13" t="s">
-        <v>99</v>
-      </c>
-      <c r="AB34" s="13">
+      <c r="Y34" s="11">
+        <v>0.01</v>
+      </c>
+      <c r="Z34" s="11">
+        <v>0.01</v>
+      </c>
+      <c r="AA34" s="11" t="s">
+        <v>57</v>
+      </c>
+      <c r="AB34" s="11">
         <v>0.85</v>
       </c>
     </row>
     <row r="35" spans="20:28">
       <c r="T35" s="2" t="s">
-        <v>96</v>
-      </c>
-      <c r="U35" s="14">
+        <v>54</v>
+      </c>
+      <c r="U35" s="12">
         <v>1.5</v>
       </c>
-      <c r="V35" s="13">
+      <c r="V35" s="11">
         <v>0.28999999999999998</v>
       </c>
-      <c r="W35" s="13">
+      <c r="W35" s="11">
         <v>0.88</v>
       </c>
-      <c r="X35" s="13">
+      <c r="X35" s="11">
         <v>0.4</v>
       </c>
-      <c r="Y35" s="13">
+      <c r="Y35" s="11">
         <v>6.0000000000000001E-3</v>
       </c>
-      <c r="Z35" s="13" t="s">
-        <v>99</v>
-      </c>
-      <c r="AA35" s="13" t="s">
-        <v>100</v>
-      </c>
-      <c r="AB35" s="13">
+      <c r="Z35" s="11" t="s">
+        <v>57</v>
+      </c>
+      <c r="AA35" s="11" t="s">
+        <v>58</v>
+      </c>
+      <c r="AB35" s="11">
         <v>0.85</v>
       </c>
     </row>
     <row r="36" spans="20:28">
       <c r="T36" s="2" t="s">
-        <v>97</v>
-      </c>
-      <c r="U36" s="14">
+        <v>55</v>
+      </c>
+      <c r="U36" s="12">
         <v>2.08</v>
       </c>
-      <c r="V36" s="13">
+      <c r="V36" s="11">
         <v>0.33</v>
       </c>
-      <c r="W36" s="13">
+      <c r="W36" s="11">
         <v>0.96</v>
       </c>
-      <c r="X36" s="13">
+      <c r="X36" s="11">
         <v>0.4</v>
       </c>
-      <c r="Y36" s="13">
+      <c r="Y36" s="11">
         <v>8.9999999999999993E-3</v>
       </c>
-      <c r="Z36" s="13">
-        <v>0.01</v>
-      </c>
-      <c r="AA36" s="13">
+      <c r="Z36" s="11">
+        <v>0.01</v>
+      </c>
+      <c r="AA36" s="11">
         <v>0.5</v>
       </c>
-      <c r="AB36" s="13">
+      <c r="AB36" s="11">
         <v>0.85</v>
       </c>
     </row>
     <row r="37" spans="20:28">
       <c r="T37" s="2" t="s">
-        <v>75</v>
-      </c>
-      <c r="U37" s="14">
+        <v>33</v>
+      </c>
+      <c r="U37" s="12">
         <v>1.34</v>
       </c>
-      <c r="V37" s="13">
+      <c r="V37" s="11">
         <v>0.37</v>
       </c>
-      <c r="W37" s="13">
+      <c r="W37" s="11">
         <v>0.88</v>
       </c>
-      <c r="X37" s="13">
+      <c r="X37" s="11">
         <v>0.4</v>
       </c>
-      <c r="Y37" s="13">
+      <c r="Y37" s="11">
         <v>6.0000000000000001E-3</v>
       </c>
-      <c r="Z37" s="13">
-        <v>0.01</v>
-      </c>
-      <c r="AA37" s="13" t="s">
-        <v>99</v>
-      </c>
-      <c r="AB37" s="13">
+      <c r="Z37" s="11">
+        <v>0.01</v>
+      </c>
+      <c r="AA37" s="11" t="s">
+        <v>57</v>
+      </c>
+      <c r="AB37" s="11">
         <v>0.85</v>
       </c>
     </row>
     <row r="38" spans="20:28">
       <c r="T38" s="2" t="s">
-        <v>113</v>
-      </c>
-      <c r="U38" s="12">
+        <v>71</v>
+      </c>
+      <c r="U38" s="10">
         <v>1</v>
       </c>
-      <c r="V38" s="12">
+      <c r="V38" s="10">
         <v>0.22</v>
       </c>
-      <c r="W38" s="12">
+      <c r="W38" s="10">
         <v>0.85</v>
       </c>
-      <c r="X38" s="12">
+      <c r="X38" s="10">
         <v>0.4</v>
       </c>
-      <c r="Y38" s="12">
+      <c r="Y38" s="10">
         <v>8.0000000000000002E-3</v>
       </c>
-      <c r="Z38" s="12">
+      <c r="Z38" s="10">
         <v>8.9999999999999993E-3</v>
       </c>
-      <c r="AA38" s="12" t="s">
-        <v>59</v>
-      </c>
-      <c r="AB38" s="12" t="s">
-        <v>99</v>
+      <c r="AA38" s="10" t="s">
+        <v>17</v>
+      </c>
+      <c r="AB38" s="10" t="s">
+        <v>57</v>
       </c>
     </row>
     <row r="39" spans="20:28">
       <c r="T39" s="2" t="s">
-        <v>102</v>
-      </c>
-      <c r="U39" s="12">
+        <v>60</v>
+      </c>
+      <c r="U39" s="10">
         <v>1.5</v>
       </c>
-      <c r="V39" s="12">
+      <c r="V39" s="10">
         <v>0.28999999999999998</v>
       </c>
-      <c r="W39" s="12">
+      <c r="W39" s="10">
         <v>0.88</v>
       </c>
-      <c r="X39" s="12">
+      <c r="X39" s="10">
         <v>0.4</v>
       </c>
-      <c r="Y39" s="12">
+      <c r="Y39" s="10">
         <v>6.0000000000000001E-3</v>
       </c>
-      <c r="Z39" s="12" t="s">
-        <v>59</v>
-      </c>
-      <c r="AA39" s="12" t="s">
-        <v>59</v>
-      </c>
-      <c r="AB39" s="12" t="s">
-        <v>99</v>
+      <c r="Z39" s="10" t="s">
+        <v>17</v>
+      </c>
+      <c r="AA39" s="10" t="s">
+        <v>17</v>
+      </c>
+      <c r="AB39" s="10" t="s">
+        <v>57</v>
       </c>
     </row>
     <row r="40" spans="20:28">
       <c r="T40" s="2"/>
-      <c r="U40" s="14"/>
-      <c r="V40" s="13"/>
-      <c r="W40" s="13"/>
-      <c r="X40" s="13"/>
-      <c r="Y40" s="13"/>
-      <c r="Z40" s="13"/>
-      <c r="AA40" s="13"/>
-      <c r="AB40" s="13"/>
+      <c r="U40" s="12"/>
+      <c r="V40" s="11"/>
+      <c r="W40" s="11"/>
+      <c r="X40" s="11"/>
+      <c r="Y40" s="11"/>
+      <c r="Z40" s="11"/>
+      <c r="AA40" s="11"/>
+      <c r="AB40" s="11"/>
     </row>
     <row r="41" spans="20:28">
       <c r="T41" s="2"/>
@@ -3030,21 +2743,21 @@
     </row>
     <row r="42" spans="20:28">
       <c r="T42" s="2" t="s">
-        <v>70</v>
+        <v>28</v>
       </c>
       <c r="U42" s="2" t="s">
-        <v>71</v>
+        <v>29</v>
       </c>
       <c r="V42" s="2" t="s">
-        <v>72</v>
+        <v>30</v>
       </c>
     </row>
     <row r="43" spans="20:28">
       <c r="T43" s="2" t="s">
-        <v>74</v>
+        <v>32</v>
       </c>
       <c r="U43" s="2" t="s">
-        <v>73</v>
+        <v>31</v>
       </c>
       <c r="V43">
         <v>0.06</v>
@@ -3052,10 +2765,10 @@
     </row>
     <row r="44" spans="20:28">
       <c r="T44" s="2" t="s">
-        <v>76</v>
+        <v>34</v>
       </c>
       <c r="U44" s="2" t="s">
-        <v>73</v>
+        <v>31</v>
       </c>
       <c r="V44">
         <v>1</v>
@@ -3063,10 +2776,10 @@
     </row>
     <row r="45" spans="20:28">
       <c r="T45" t="s">
-        <v>11</v>
+        <v>3</v>
       </c>
       <c r="U45" s="2" t="s">
-        <v>73</v>
+        <v>31</v>
       </c>
       <c r="V45">
         <v>0</v>
@@ -3074,10 +2787,10 @@
     </row>
     <row r="46" spans="20:28">
       <c r="T46" s="2" t="s">
-        <v>96</v>
+        <v>54</v>
       </c>
       <c r="U46" s="2" t="s">
-        <v>73</v>
+        <v>31</v>
       </c>
       <c r="V46">
         <v>0</v>
@@ -3085,10 +2798,10 @@
     </row>
     <row r="47" spans="20:28">
       <c r="T47" s="2" t="s">
-        <v>75</v>
+        <v>33</v>
       </c>
       <c r="U47" s="2" t="s">
-        <v>73</v>
+        <v>31</v>
       </c>
       <c r="V47">
         <v>0.8</v>
@@ -3096,10 +2809,10 @@
     </row>
     <row r="48" spans="20:28">
       <c r="T48" s="2" t="s">
-        <v>82</v>
+        <v>40</v>
       </c>
       <c r="U48" s="2" t="s">
-        <v>77</v>
+        <v>35</v>
       </c>
       <c r="V48">
         <v>0</v>
@@ -3107,10 +2820,10 @@
     </row>
     <row r="49" spans="20:22">
       <c r="T49" s="2" t="s">
-        <v>82</v>
+        <v>40</v>
       </c>
       <c r="U49" s="2" t="s">
-        <v>78</v>
+        <v>36</v>
       </c>
       <c r="V49">
         <v>0.03</v>
@@ -3118,10 +2831,10 @@
     </row>
     <row r="50" spans="20:22">
       <c r="T50" s="2" t="s">
-        <v>82</v>
+        <v>40</v>
       </c>
       <c r="U50" s="2" t="s">
-        <v>79</v>
+        <v>37</v>
       </c>
       <c r="V50">
         <v>0</v>
@@ -3129,10 +2842,10 @@
     </row>
     <row r="51" spans="20:22">
       <c r="T51" s="2" t="s">
-        <v>81</v>
+        <v>39</v>
       </c>
       <c r="U51" s="2" t="s">
-        <v>77</v>
+        <v>35</v>
       </c>
       <c r="V51">
         <v>0.05</v>
@@ -3140,10 +2853,10 @@
     </row>
     <row r="52" spans="20:22">
       <c r="T52" s="2" t="s">
-        <v>81</v>
+        <v>39</v>
       </c>
       <c r="U52" s="2" t="s">
-        <v>80</v>
+        <v>38</v>
       </c>
       <c r="V52">
         <v>7.0000000000000007E-2</v>
@@ -3151,10 +2864,10 @@
     </row>
     <row r="53" spans="20:22">
       <c r="T53" s="2" t="s">
-        <v>81</v>
+        <v>39</v>
       </c>
       <c r="U53" s="2" t="s">
-        <v>78</v>
+        <v>36</v>
       </c>
       <c r="V53">
         <v>0.04</v>
@@ -3162,10 +2875,10 @@
     </row>
     <row r="54" spans="20:22">
       <c r="T54" s="2" t="s">
-        <v>81</v>
+        <v>39</v>
       </c>
       <c r="U54" s="2" t="s">
-        <v>101</v>
+        <v>59</v>
       </c>
       <c r="V54">
         <v>0.09</v>
@@ -3173,10 +2886,10 @@
     </row>
     <row r="55" spans="20:22">
       <c r="T55" s="2" t="s">
-        <v>81</v>
+        <v>39</v>
       </c>
       <c r="U55" s="2" t="s">
-        <v>79</v>
+        <v>37</v>
       </c>
       <c r="V55">
         <v>0.11</v>
@@ -3184,10 +2897,10 @@
     </row>
     <row r="56" spans="20:22">
       <c r="T56" s="2" t="s">
-        <v>81</v>
+        <v>39</v>
       </c>
       <c r="U56" s="2" t="s">
-        <v>104</v>
+        <v>62</v>
       </c>
       <c r="V56">
         <v>0.16</v>
@@ -3195,10 +2908,10 @@
     </row>
     <row r="57" spans="20:22">
       <c r="T57" s="2" t="s">
-        <v>81</v>
+        <v>39</v>
       </c>
       <c r="U57" s="2" t="s">
-        <v>105</v>
+        <v>63</v>
       </c>
       <c r="V57">
         <v>0.01</v>
@@ -3206,10 +2919,10 @@
     </row>
     <row r="58" spans="20:22">
       <c r="T58" s="2" t="s">
-        <v>81</v>
+        <v>39</v>
       </c>
       <c r="U58" s="2" t="s">
-        <v>103</v>
+        <v>61</v>
       </c>
       <c r="V58">
         <v>0</v>
@@ -3219,576 +2932,4 @@
   <dataConsolidate/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
-</file>
-
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C262A7CE-34CD-7A40-9BF6-875F02812705}">
-  <dimension ref="A1:P46"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="16"/>
-  <cols>
-    <col min="1" max="1" width="31" style="3" customWidth="1"/>
-    <col min="2" max="3" width="26.6640625" customWidth="1"/>
-    <col min="5" max="5" width="16" customWidth="1"/>
-    <col min="6" max="7" width="16.5" customWidth="1"/>
-    <col min="8" max="8" width="12.83203125" customWidth="1"/>
-    <col min="10" max="10" width="12.1640625" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="36" customWidth="1"/>
-    <col min="16" max="16" width="28.5" style="10" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:13" ht="17">
-      <c r="A1" s="3" t="s">
-        <v>0</v>
-      </c>
-      <c r="J1" s="1" t="s">
-        <v>39</v>
-      </c>
-    </row>
-    <row r="2" spans="1:13">
-      <c r="H2" s="1" t="s">
-        <v>40</v>
-      </c>
-      <c r="J2" s="1"/>
-    </row>
-    <row r="3" spans="1:13">
-      <c r="C3" t="s">
-        <v>35</v>
-      </c>
-      <c r="F3" t="s">
-        <v>44</v>
-      </c>
-      <c r="J3" s="1"/>
-    </row>
-    <row r="4" spans="1:13" ht="17">
-      <c r="A4" s="4" t="s">
-        <v>22</v>
-      </c>
-      <c r="B4" s="5" t="s">
-        <v>18</v>
-      </c>
-      <c r="C4" s="5" t="s">
-        <v>19</v>
-      </c>
-      <c r="D4" t="s">
-        <v>20</v>
-      </c>
-      <c r="E4" s="5" t="s">
-        <v>21</v>
-      </c>
-      <c r="F4" t="s">
-        <v>43</v>
-      </c>
-      <c r="G4" s="9"/>
-      <c r="H4" t="s">
-        <v>41</v>
-      </c>
-      <c r="I4" t="s">
-        <v>17</v>
-      </c>
-      <c r="J4" s="6" t="s">
-        <v>45</v>
-      </c>
-      <c r="L4" s="7" t="s">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="5" spans="1:13">
-      <c r="A5" s="2"/>
-      <c r="H5" t="str">
-        <f>IF(ISBLANK(A5), "", F5*$M$9)</f>
-        <v/>
-      </c>
-      <c r="I5" t="str">
-        <f>IF(ISBLANK(A5),"",VLOOKUP(B5,L14:M28,2,FALSE))</f>
-        <v/>
-      </c>
-      <c r="J5" t="str">
-        <f>IF(ISBLANK(A5), "", H5*I5*$M$10/1000)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="6" spans="1:13">
-      <c r="H6" t="str">
-        <f t="shared" ref="H6:H11" si="0">IF(ISBLANK(A6), "", F6*G6)</f>
-        <v/>
-      </c>
-      <c r="I6" t="str">
-        <f t="shared" ref="I6:I16" si="1">IF(ISBLANK(A6),"",VLOOKUP(B6,L15:M29,2,FALSE))</f>
-        <v/>
-      </c>
-      <c r="J6" t="str">
-        <f t="shared" ref="J6:J16" si="2">IF(ISBLANK(A6), "", H6*I6*$M$10/1000)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="7" spans="1:13">
-      <c r="B7" s="2"/>
-      <c r="H7" t="str">
-        <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="I7" t="str">
-        <f>IF(ISBLANK(A9),"",VLOOKUP(B7,L16:M30,2,FALSE))</f>
-        <v/>
-      </c>
-      <c r="J7" t="str">
-        <f>IF(ISBLANK(A9), "", H7*I7*$M$10/1000)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="8" spans="1:13">
-      <c r="A8" s="2"/>
-      <c r="B8" s="2"/>
-      <c r="H8" t="str">
-        <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="I8" t="str">
-        <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="J8" t="str">
-        <f t="shared" si="2"/>
-        <v/>
-      </c>
-      <c r="L8" s="2"/>
-      <c r="M8" s="2"/>
-    </row>
-    <row r="9" spans="1:13">
-      <c r="A9" s="2"/>
-      <c r="B9" s="2"/>
-      <c r="H9" t="str">
-        <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="I9" t="str">
-        <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="J9" t="str">
-        <f t="shared" si="2"/>
-        <v/>
-      </c>
-      <c r="L9" s="11" t="s">
-        <v>42</v>
-      </c>
-      <c r="M9" s="2">
-        <v>0.21</v>
-      </c>
-    </row>
-    <row r="10" spans="1:13">
-      <c r="A10" s="2"/>
-      <c r="B10" s="2"/>
-      <c r="H10" t="str">
-        <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="I10" t="str">
-        <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="J10" t="str">
-        <f t="shared" si="2"/>
-        <v/>
-      </c>
-      <c r="L10" t="s">
-        <v>2</v>
-      </c>
-      <c r="M10">
-        <f>44/28</f>
-        <v>1.5714285714285714</v>
-      </c>
-    </row>
-    <row r="11" spans="1:13">
-      <c r="A11" s="2"/>
-      <c r="B11" s="2"/>
-      <c r="H11" t="str">
-        <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="L11" s="2"/>
-      <c r="M11" s="2"/>
-    </row>
-    <row r="12" spans="1:13">
-      <c r="F12" t="str">
-        <f t="shared" ref="F6:F16" si="3">IF(ISBLANK(A12), "", IF(ISNUMBER(E12), E12*C12, D12*C12))</f>
-        <v/>
-      </c>
-      <c r="L12" s="2" t="s">
-        <v>17</v>
-      </c>
-      <c r="M12" s="2"/>
-    </row>
-    <row r="13" spans="1:13">
-      <c r="A13" s="2"/>
-      <c r="F13" t="str">
-        <f t="shared" si="3"/>
-        <v/>
-      </c>
-      <c r="G13" t="str">
-        <f t="shared" ref="G13:G16" si="4">IF(ISBLANK(A13), "", VLOOKUP(A13, L41:N47, 3, FALSE))</f>
-        <v/>
-      </c>
-      <c r="H13" t="str">
-        <f t="shared" ref="H13:H16" si="5">IF(ISBLANK(A13), "", F13*G13)</f>
-        <v/>
-      </c>
-      <c r="I13" t="str">
-        <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="J13" t="str">
-        <f t="shared" si="2"/>
-        <v/>
-      </c>
-      <c r="L13" t="s">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="14" spans="1:13">
-      <c r="A14" s="2"/>
-      <c r="F14" t="str">
-        <f t="shared" si="3"/>
-        <v/>
-      </c>
-      <c r="G14" t="str">
-        <f t="shared" si="4"/>
-        <v/>
-      </c>
-      <c r="H14" t="str">
-        <f t="shared" si="5"/>
-        <v/>
-      </c>
-      <c r="I14" t="str">
-        <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="J14" t="str">
-        <f t="shared" si="2"/>
-        <v/>
-      </c>
-      <c r="L14" s="2" t="s">
-        <v>4</v>
-      </c>
-      <c r="M14" s="2">
-        <v>5.8999999999999999E-3</v>
-      </c>
-    </row>
-    <row r="15" spans="1:13">
-      <c r="A15" s="2"/>
-      <c r="B15" s="2"/>
-      <c r="F15" t="str">
-        <f t="shared" si="3"/>
-        <v/>
-      </c>
-      <c r="G15" t="str">
-        <f t="shared" si="4"/>
-        <v/>
-      </c>
-      <c r="H15" t="str">
-        <f t="shared" si="5"/>
-        <v/>
-      </c>
-      <c r="I15" t="str">
-        <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="J15" t="str">
-        <f t="shared" si="2"/>
-        <v/>
-      </c>
-      <c r="L15" s="2" t="s">
-        <v>5</v>
-      </c>
-      <c r="M15" s="2">
-        <v>2.8999999999999998E-3</v>
-      </c>
-    </row>
-    <row r="16" spans="1:13">
-      <c r="B16" s="2"/>
-      <c r="F16" t="str">
-        <f t="shared" si="3"/>
-        <v/>
-      </c>
-      <c r="G16" t="str">
-        <f t="shared" si="4"/>
-        <v/>
-      </c>
-      <c r="H16" t="str">
-        <f t="shared" si="5"/>
-        <v/>
-      </c>
-      <c r="I16" t="str">
-        <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="J16" t="str">
-        <f t="shared" si="2"/>
-        <v/>
-      </c>
-      <c r="L16" s="2" t="s">
-        <v>6</v>
-      </c>
-      <c r="M16" s="2">
-        <v>8.0000000000000002E-3</v>
-      </c>
-    </row>
-    <row r="17" spans="2:13">
-      <c r="L17" s="2" t="s">
-        <v>7</v>
-      </c>
-      <c r="M17" s="2">
-        <v>7.0000000000000001E-3</v>
-      </c>
-    </row>
-    <row r="18" spans="2:13">
-      <c r="L18" s="2" t="s">
-        <v>8</v>
-      </c>
-      <c r="M18" s="2">
-        <v>1.8E-3</v>
-      </c>
-    </row>
-    <row r="19" spans="2:13">
-      <c r="L19" s="2" t="s">
-        <v>9</v>
-      </c>
-      <c r="M19" s="2">
-        <v>4.1000000000000003E-3</v>
-      </c>
-    </row>
-    <row r="20" spans="2:13">
-      <c r="L20" s="2" t="s">
-        <v>10</v>
-      </c>
-      <c r="M20" s="2">
-        <v>1.9900000000000001E-2</v>
-      </c>
-    </row>
-    <row r="21" spans="2:13">
-      <c r="B21" s="2"/>
-      <c r="L21" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="M21" s="2">
-        <v>5.3E-3</v>
-      </c>
-    </row>
-    <row r="22" spans="2:13">
-      <c r="B22" s="2"/>
-      <c r="L22" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="M22" s="2">
-        <v>6.4000000000000003E-3</v>
-      </c>
-    </row>
-    <row r="23" spans="2:13">
-      <c r="H23" t="str">
-        <f t="shared" ref="H23:H26" si="6">IF(ISBLANK(C23), "", D23/C23)</f>
-        <v/>
-      </c>
-      <c r="L23" s="2" t="s">
-        <v>13</v>
-      </c>
-      <c r="M23" s="2">
-        <v>2.5999999999999999E-3</v>
-      </c>
-    </row>
-    <row r="24" spans="2:13">
-      <c r="H24" t="str">
-        <f t="shared" si="6"/>
-        <v/>
-      </c>
-      <c r="L24" s="2" t="s">
-        <v>14</v>
-      </c>
-      <c r="M24" s="2">
-        <v>3.0000000000000001E-3</v>
-      </c>
-    </row>
-    <row r="25" spans="2:13">
-      <c r="H25" t="str">
-        <f t="shared" si="6"/>
-        <v/>
-      </c>
-      <c r="L25" s="2" t="s">
-        <v>15</v>
-      </c>
-      <c r="M25" s="8">
-        <v>5.0000000000000001E-3</v>
-      </c>
-    </row>
-    <row r="26" spans="2:13">
-      <c r="H26" t="str">
-        <f t="shared" si="6"/>
-        <v/>
-      </c>
-      <c r="L26" s="2"/>
-      <c r="M26" s="8"/>
-    </row>
-    <row r="27" spans="2:13">
-      <c r="L27" s="2" t="s">
-        <v>13</v>
-      </c>
-      <c r="M27" s="2">
-        <v>2.5999999999999999E-3</v>
-      </c>
-    </row>
-    <row r="28" spans="2:13">
-      <c r="L28" s="2" t="s">
-        <v>16</v>
-      </c>
-      <c r="M28" s="2">
-        <v>1.8E-3</v>
-      </c>
-    </row>
-    <row r="29" spans="2:13">
-      <c r="L29" s="2"/>
-      <c r="M29" s="2"/>
-    </row>
-    <row r="30" spans="2:13">
-      <c r="L30" s="2"/>
-      <c r="M30" s="2"/>
-    </row>
-    <row r="31" spans="2:13">
-      <c r="L31" s="2"/>
-      <c r="M31" s="2"/>
-    </row>
-    <row r="32" spans="2:13">
-      <c r="L32" s="2" t="s">
-        <v>23</v>
-      </c>
-    </row>
-    <row r="33" spans="12:16">
-      <c r="L33" s="2" t="s">
-        <v>24</v>
-      </c>
-      <c r="M33" s="2">
-        <v>0.1</v>
-      </c>
-      <c r="N33">
-        <v>0.08</v>
-      </c>
-    </row>
-    <row r="34" spans="12:16" ht="51">
-      <c r="L34" s="2" t="s">
-        <v>25</v>
-      </c>
-      <c r="M34" s="2">
-        <v>0.18</v>
-      </c>
-      <c r="N34">
-        <v>0.08</v>
-      </c>
-      <c r="P34" s="10" t="s">
-        <v>36</v>
-      </c>
-    </row>
-    <row r="35" spans="12:16">
-      <c r="L35" s="2" t="s">
-        <v>26</v>
-      </c>
-      <c r="M35" s="2">
-        <v>0.46</v>
-      </c>
-      <c r="N35">
-        <v>0.15</v>
-      </c>
-    </row>
-    <row r="36" spans="12:16">
-      <c r="L36" s="2" t="s">
-        <v>27</v>
-      </c>
-      <c r="M36" s="2">
-        <v>0.21</v>
-      </c>
-      <c r="N36">
-        <v>0.08</v>
-      </c>
-    </row>
-    <row r="37" spans="12:16">
-      <c r="L37" s="2" t="s">
-        <v>38</v>
-      </c>
-      <c r="M37" s="2">
-        <v>0.32</v>
-      </c>
-      <c r="N37">
-        <v>0.05</v>
-      </c>
-    </row>
-    <row r="38" spans="12:16">
-      <c r="L38" s="2" t="s">
-        <v>28</v>
-      </c>
-      <c r="M38" s="2">
-        <v>0.33700000000000002</v>
-      </c>
-      <c r="N38">
-        <v>0.05</v>
-      </c>
-    </row>
-    <row r="39" spans="12:16">
-      <c r="L39" s="2" t="s">
-        <v>37</v>
-      </c>
-      <c r="M39" s="2">
-        <v>0.27</v>
-      </c>
-      <c r="N39">
-        <v>0.05</v>
-      </c>
-    </row>
-    <row r="41" spans="12:16">
-      <c r="L41" s="2" t="s">
-        <v>34</v>
-      </c>
-    </row>
-    <row r="42" spans="12:16">
-      <c r="L42" s="2" t="s">
-        <v>29</v>
-      </c>
-      <c r="M42" s="2">
-        <v>0.15</v>
-      </c>
-    </row>
-    <row r="43" spans="12:16">
-      <c r="L43" s="2" t="s">
-        <v>30</v>
-      </c>
-      <c r="M43" s="2">
-        <v>0.08</v>
-      </c>
-    </row>
-    <row r="44" spans="12:16">
-      <c r="L44" s="2" t="s">
-        <v>31</v>
-      </c>
-      <c r="M44" s="2">
-        <v>0.01</v>
-      </c>
-    </row>
-    <row r="45" spans="12:16">
-      <c r="L45" s="2" t="s">
-        <v>32</v>
-      </c>
-      <c r="M45" s="2">
-        <v>0.05</v>
-      </c>
-    </row>
-    <row r="46" spans="12:16">
-      <c r="L46" s="2" t="s">
-        <v>33</v>
-      </c>
-      <c r="M46" s="2">
-        <v>0.11</v>
-      </c>
-    </row>
-  </sheetData>
-  <mergeCells count="1">
-    <mergeCell ref="M25:M26"/>
-  </mergeCells>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
 </file>
</xml_diff>